<commit_message>
Excel-Berichte: WebGIS-Eigentümer nach ihrem Typ zählen und färben
Seit das Holen den Eigentümer wie im WebGIS setzt, stehen dort Namen wie
«AWU_von_privat» oder an der Haltung «Altdorf (Gemeinde)». Die Vorlagen
verglichen nur «Abwasser Uri», «AWU», «Kanton Uri», «Kanton», «Bund»,
«Gemeinde» und «Privat» exakt, deshalb blieben diese Zeilen ungefärbt und
fehlten in «Kosten nach Eigentümer» (Entscheid Pascal 24.09.2026: ja).

Jeder WebGIS-Name zählt, summiert und färbt jetzt nach seinem WebGIS-Typ in
der bestehenden Kategorie: Abwasserverband wie Abwasser Uri, dazu Kanton,
Bund, Gemeinde und Privat. Genossenschaften und «Unbekannt» bleiben wie bisher
ungefärbt. Der Vorlagenbauer und ExcelReportStyle.Eigentuemer lesen dieselbe
Liste aus dem Objektaktenkatalog. Neu gebaut mit openpyxl 3.1.5 und
Pillow 11.3.0; ohne Änderung war der Nachbau bis auf docProps/core.xml
identisch mit den bisherigen Vorlagen.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Export_Vorlage/Haltungen.xlsx
+++ b/Export_Vorlage/Haltungen.xlsx
@@ -2636,7 +2636,7 @@
         </is>
       </c>
       <c r="E17" s="12">
-        <f>COUNTIF('Haltungen'!$O$27:$O$5000,"Abwasser Uri")+COUNTIF('Haltungen'!$O$27:$O$5000,"AWU")</f>
+        <f>COUNTIF('Haltungen'!$O$27:$O$5000,"Abwasser Uri")+COUNTIF('Haltungen'!$O$27:$O$5000,"AWU")+COUNTIF('Haltungen'!$O$27:$O$5000,"AWU_von_oeffentlich")+COUNTIF('Haltungen'!$O$27:$O$5000,"AWU_von_oeffentlich (Abwasserverband)")+COUNTIF('Haltungen'!$O$27:$O$5000,"AWU_von_privat")+COUNTIF('Haltungen'!$O$27:$O$5000,"AWU_von_privat (Abwasserverband)")</f>
         <v/>
       </c>
       <c r="F17" s="14" t="inlineStr">
@@ -2684,7 +2684,7 @@
       <c r="P17" s="2" t="n"/>
       <c r="Q17" s="2" t="n"/>
       <c r="R17" s="17">
-        <f>SUMIF('Haltungen'!$O$27:$O$5000,"Abwasser Uri",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"AWU",'Haltungen'!$N$27:$N$5000)</f>
+        <f>SUMIF('Haltungen'!$O$27:$O$5000,"Abwasser Uri",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"AWU",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"AWU_von_oeffentlich",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"AWU_von_oeffentlich (Abwasserverband)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"AWU_von_privat",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"AWU_von_privat (Abwasserverband)",'Haltungen'!$N$27:$N$5000)</f>
         <v/>
       </c>
       <c r="S17" s="16" t="inlineStr">
@@ -2728,7 +2728,7 @@
         </is>
       </c>
       <c r="E18" s="12">
-        <f>COUNTIF('Haltungen'!$O$27:$O$5000,"Kanton Uri")+COUNTIF('Haltungen'!$O$27:$O$5000,"Kanton")</f>
+        <f>COUNTIF('Haltungen'!$O$27:$O$5000,"Kanton Uri")+COUNTIF('Haltungen'!$O$27:$O$5000,"Kanton")+COUNTIF('Haltungen'!$O$27:$O$5000,"Kanton Uri (Kanton)")</f>
         <v/>
       </c>
       <c r="F18" s="21" t="inlineStr">
@@ -2776,7 +2776,7 @@
       <c r="P18" s="2" t="n"/>
       <c r="Q18" s="2" t="n"/>
       <c r="R18" s="17">
-        <f>SUMIF('Haltungen'!$O$27:$O$5000,"Kanton Uri",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Kanton",'Haltungen'!$N$27:$N$5000)</f>
+        <f>SUMIF('Haltungen'!$O$27:$O$5000,"Kanton Uri",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Kanton",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Kanton Uri (Kanton)",'Haltungen'!$N$27:$N$5000)</f>
         <v/>
       </c>
       <c r="S18" s="16" t="inlineStr">
@@ -2820,7 +2820,7 @@
         </is>
       </c>
       <c r="E19" s="12">
-        <f>COUNTIF('Haltungen'!$O$27:$O$5000,"Bund")</f>
+        <f>COUNTIF('Haltungen'!$O$27:$O$5000,"Bund")+COUNTIF('Haltungen'!$O$27:$O$5000,"Bund Astra")+COUNTIF('Haltungen'!$O$27:$O$5000,"Bund Astra (Bund)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Bund (Bund)")</f>
         <v/>
       </c>
       <c r="F19" s="26" t="inlineStr">
@@ -2861,7 +2861,7 @@
       <c r="P19" s="2" t="n"/>
       <c r="Q19" s="2" t="n"/>
       <c r="R19" s="17">
-        <f>SUMIF('Haltungen'!$O$27:$O$5000,"Bund",'Haltungen'!$N$27:$N$5000)</f>
+        <f>SUMIF('Haltungen'!$O$27:$O$5000,"Bund",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Bund Astra",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Bund Astra (Bund)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Bund (Bund)",'Haltungen'!$N$27:$N$5000)</f>
         <v/>
       </c>
       <c r="S19" s="16" t="inlineStr">
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="E20" s="12">
-        <f>COUNTIF('Haltungen'!$O$27:$O$5000,"Gemeinde")</f>
+        <f>COUNTIF('Haltungen'!$O$27:$O$5000,"Gemeinde")+COUNTIF('Haltungen'!$O$27:$O$5000,"Altdorf")+COUNTIF('Haltungen'!$O$27:$O$5000,"Altdorf (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Bürglen")+COUNTIF('Haltungen'!$O$27:$O$5000,"Bürglen (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Schattdorf")+COUNTIF('Haltungen'!$O$27:$O$5000,"Schattdorf (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Andermatt")+COUNTIF('Haltungen'!$O$27:$O$5000,"Andermatt (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Attinghausen")+COUNTIF('Haltungen'!$O$27:$O$5000,"Attinghausen (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Erstfeld")+COUNTIF('Haltungen'!$O$27:$O$5000,"Erstfeld (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Flüelen")+COUNTIF('Haltungen'!$O$27:$O$5000,"Flüelen (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Göschenen")+COUNTIF('Haltungen'!$O$27:$O$5000,"Göschenen (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Gurtnellen")+COUNTIF('Haltungen'!$O$27:$O$5000,"Gurtnellen (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Hospental")+COUNTIF('Haltungen'!$O$27:$O$5000,"Hospental (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Isenthal")+COUNTIF('Haltungen'!$O$27:$O$5000,"Isenthal (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Realp")+COUNTIF('Haltungen'!$O$27:$O$5000,"Realp (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Seedorf")+COUNTIF('Haltungen'!$O$27:$O$5000,"Seedorf (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Seelisberg")+COUNTIF('Haltungen'!$O$27:$O$5000,"Seelisberg (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Silenen")+COUNTIF('Haltungen'!$O$27:$O$5000,"Silenen (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Sisikon")+COUNTIF('Haltungen'!$O$27:$O$5000,"Sisikon (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Spiringen")+COUNTIF('Haltungen'!$O$27:$O$5000,"Spiringen (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Unterschächen")+COUNTIF('Haltungen'!$O$27:$O$5000,"Unterschächen (Gemeinde)")+COUNTIF('Haltungen'!$O$27:$O$5000,"Wassen")+COUNTIF('Haltungen'!$O$27:$O$5000,"Wassen (Gemeinde)")</f>
         <v/>
       </c>
       <c r="F20" s="19" t="inlineStr">
@@ -2946,7 +2946,7 @@
       <c r="P20" s="2" t="n"/>
       <c r="Q20" s="2" t="n"/>
       <c r="R20" s="17">
-        <f>SUMIF('Haltungen'!$O$27:$O$5000,"Gemeinde",'Haltungen'!$N$27:$N$5000)</f>
+        <f>SUMIF('Haltungen'!$O$27:$O$5000,"Gemeinde",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Altdorf",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Altdorf (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Bürglen",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Bürglen (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Schattdorf",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Schattdorf (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Andermatt",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Andermatt (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Attinghausen",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Attinghausen (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Erstfeld",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Erstfeld (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Flüelen",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Flüelen (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Göschenen",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Göschenen (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Gurtnellen",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Gurtnellen (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Hospental",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Hospental (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Isenthal",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Isenthal (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Realp",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Realp (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Seedorf",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Seedorf (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Seelisberg",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Seelisberg (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Silenen",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Silenen (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Sisikon",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Sisikon (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Spiringen",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Spiringen (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Unterschächen",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Unterschächen (Gemeinde)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Wassen",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Wassen (Gemeinde)",'Haltungen'!$N$27:$N$5000)</f>
         <v/>
       </c>
       <c r="S20" s="16" t="inlineStr">
@@ -2983,7 +2983,7 @@
         </is>
       </c>
       <c r="E21" s="12">
-        <f>COUNTIF('Haltungen'!$O$27:$O$5000,"Privat")</f>
+        <f>COUNTIF('Haltungen'!$O$27:$O$5000,"Privat")+COUNTIF('Haltungen'!$O$27:$O$5000,"Privat (Privat)")+COUNTIF('Haltungen'!$O$27:$O$5000,"RUAG")+COUNTIF('Haltungen'!$O$27:$O$5000,"RUAG (Privat)")</f>
         <v/>
       </c>
       <c r="F21" s="31" t="inlineStr">
@@ -3017,7 +3017,7 @@
       <c r="P21" s="2" t="n"/>
       <c r="Q21" s="2" t="n"/>
       <c r="R21" s="17">
-        <f>SUMIF('Haltungen'!$O$27:$O$5000,"Privat",'Haltungen'!$N$27:$N$5000)</f>
+        <f>SUMIF('Haltungen'!$O$27:$O$5000,"Privat",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"Privat (Privat)",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"RUAG",'Haltungen'!$N$27:$N$5000)+SUMIF('Haltungen'!$O$27:$O$5000,"RUAG (Privat)",'Haltungen'!$N$27:$N$5000)</f>
         <v/>
       </c>
       <c r="S21" s="16" t="inlineStr">
@@ -3552,32 +3552,179 @@
     <cfRule type="expression" priority="27" dxfId="0" stopIfTrue="1">
       <formula>$O27="AWU"</formula>
     </cfRule>
-    <cfRule type="expression" priority="28" dxfId="6" stopIfTrue="1">
+    <cfRule type="expression" priority="28" dxfId="0" stopIfTrue="1">
+      <formula>$O27="AWU_von_oeffentlich"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="29" dxfId="0" stopIfTrue="1">
+      <formula>$O27="AWU_von_oeffentlich (Abwasserverband)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="30" dxfId="0" stopIfTrue="1">
+      <formula>$O27="AWU_von_privat"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="31" dxfId="0" stopIfTrue="1">
+      <formula>$O27="AWU_von_privat (Abwasserverband)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="32" dxfId="6" stopIfTrue="1">
       <formula>$O27="Kanton Uri"</formula>
     </cfRule>
-    <cfRule type="expression" priority="29" dxfId="6" stopIfTrue="1">
+    <cfRule type="expression" priority="33" dxfId="6" stopIfTrue="1">
       <formula>$O27="Kanton"</formula>
     </cfRule>
-    <cfRule type="expression" priority="30" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="34" dxfId="6" stopIfTrue="1">
+      <formula>$O27="Kanton Uri (Kanton)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="35" dxfId="10" stopIfTrue="1">
       <formula>$O27="Bund"</formula>
     </cfRule>
-    <cfRule type="expression" priority="31" dxfId="2" stopIfTrue="1">
+    <cfRule type="expression" priority="36" dxfId="10" stopIfTrue="1">
+      <formula>$O27="Bund Astra"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="37" dxfId="10" stopIfTrue="1">
+      <formula>$O27="Bund Astra (Bund)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="38" dxfId="10" stopIfTrue="1">
+      <formula>$O27="Bund (Bund)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="39" dxfId="2" stopIfTrue="1">
       <formula>$O27="Gemeinde"</formula>
     </cfRule>
-    <cfRule type="expression" priority="32" dxfId="4" stopIfTrue="1">
+    <cfRule type="expression" priority="40" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Altdorf"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="41" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Altdorf (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="42" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Bürglen"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="43" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Bürglen (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="44" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Schattdorf"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="45" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Schattdorf (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="46" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Andermatt"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="47" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Andermatt (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="48" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Attinghausen"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="49" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Attinghausen (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="50" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Erstfeld"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="51" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Erstfeld (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="52" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Flüelen"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="53" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Flüelen (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="54" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Göschenen"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="55" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Göschenen (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="56" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Gurtnellen"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="57" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Gurtnellen (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="58" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Hospental"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="59" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Hospental (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="60" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Isenthal"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="61" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Isenthal (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="62" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Realp"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="63" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Realp (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="64" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Seedorf"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="65" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Seedorf (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="66" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Seelisberg"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="67" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Seelisberg (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="68" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Silenen"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="69" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Silenen (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="70" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Sisikon"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="71" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Sisikon (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="72" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Spiringen"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="73" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Spiringen (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="74" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Unterschächen"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="75" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Unterschächen (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="76" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Wassen"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="77" dxfId="2" stopIfTrue="1">
+      <formula>$O27="Wassen (Gemeinde)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="78" dxfId="4" stopIfTrue="1">
       <formula>$O27="Privat"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="79" dxfId="4" stopIfTrue="1">
+      <formula>$O27="Privat (Privat)"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="80" dxfId="4" stopIfTrue="1">
+      <formula>$O27="RUAG"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="81" dxfId="4" stopIfTrue="1">
+      <formula>$O27="RUAG (Privat)"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z27:Z5000">
-    <cfRule type="expression" priority="33" dxfId="4" stopIfTrue="1">
+    <cfRule type="expression" priority="82" dxfId="4" stopIfTrue="1">
       <formula>$Z27="offen"</formula>
     </cfRule>
-    <cfRule type="expression" priority="34" dxfId="11" stopIfTrue="1">
+    <cfRule type="expression" priority="83" dxfId="11" stopIfTrue="1">
       <formula>$Z27="abgeschlossen"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A27:AA5000">
-    <cfRule type="expression" priority="35" dxfId="12">
+    <cfRule type="expression" priority="84" dxfId="12">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>